<commit_message>
Curly-infix: a brace of one operator reads head-first; the operators as a vocabulary (D262)
{0.3 <= $value <= 0.7} reads as the command {<= 0.3 $value 0.7}: a brace of
an odd number of nodes whose odd slots hold one bare operator, with a
number, variable, property or command among its operands. One operator a
brace; malformed infix is an error at the brace. The array remembers it
was written infix, so printing gives the spelling back. + - * fold over
two numbers or more, comparisons chain, += -= *= /= store, and a
[property] argument is evaluated for a function of one overload.
read_structure applies the rule. The repository's objectives, unlocks and
examples are rewritten infix; the stacks' results are unchanged byte for
byte. No ternary, and no && || !.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0187bvpo3FrXsxvC9SFKdms1
</commit_message>
<xml_diff>
--- a/stacks/ledger/economy.xlsx
+++ b/stacks/ledger/economy.xlsx
@@ -720,7 +720,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{&gt;= {econ.total_earned} 1500}</t>
+          <t>{{econ.total_earned} &gt;= 1500}</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{&gt;= {econ.total_earned} 4000}</t>
+          <t>{{econ.total_earned} &gt;= 4000}</t>
         </is>
       </c>
     </row>
@@ -772,7 +772,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{&gt;= {econ.total_earned} 10000}</t>
+          <t>{{econ.total_earned} &gt;= 10000}</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{&gt;= {econ.total_earned} 25000}</t>
+          <t>{{econ.total_earned} &gt;= 25000}</t>
         </is>
       </c>
     </row>

</xml_diff>